<commit_message>
update code by 17rst
</commit_message>
<xml_diff>
--- a/doc/개발진척.xlsx
+++ b/doc/개발진척.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jkjus\Documents\GitHub\school_free_time\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\GitHub\school_free_time\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8B94136-9558-4254-B074-A86BC741D9A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24E2F757-6A28-4AD7-86B6-EEF84E9A3D97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="59">
   <si>
     <t>서비스</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -672,14 +672,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F23"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="12.296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="60.59765625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.59765625" customWidth="1"/>
+    <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="60.58203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.58203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -699,7 +699,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>20</v>
       </c>
@@ -719,7 +719,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -733,7 +733,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>22</v>
       </c>
@@ -747,7 +747,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>23</v>
       </c>
@@ -764,7 +764,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>36</v>
       </c>
@@ -784,7 +784,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>24</v>
       </c>
@@ -804,7 +804,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -818,7 +818,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>26</v>
       </c>
@@ -832,7 +832,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
         <v>27</v>
       </c>
@@ -852,7 +852,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>28</v>
       </c>
@@ -866,7 +866,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>29</v>
       </c>
@@ -880,7 +880,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>30</v>
       </c>
@@ -894,7 +894,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>31</v>
       </c>
@@ -908,7 +908,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>32</v>
       </c>
@@ -922,7 +922,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>34</v>
       </c>
@@ -936,7 +936,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>39</v>
       </c>
@@ -950,7 +950,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>43</v>
       </c>
@@ -967,7 +967,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>46</v>
       </c>
@@ -981,7 +981,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>48</v>
       </c>
@@ -998,7 +998,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>51</v>
       </c>
@@ -1014,8 +1014,11 @@
       <c r="E21" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="F21" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>53</v>
       </c>
@@ -1029,7 +1032,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>56</v>
       </c>

</xml_diff>